<commit_message>
Anomalies SF1-ECU — 25/09/2026
</commit_message>
<xml_diff>
--- a/presentation/SF1-ECU/anomalies.xlsx
+++ b/presentation/SF1-ECU/anomalies.xlsx
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U9"/>
+  <dimension ref="A1:U34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1109,36 +1109,36 @@
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>13737023</v>
+        <v>13736951</v>
       </c>
       <c r="B8" t="n">
-        <v>4002815925</v>
+        <v>4002815812</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Contrôle moteur MT en marche</t>
+          <t>Entretien systé salle électriq</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>OR004002815925</t>
+          <t>OR004002815812</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>SF01-UT-0PEM-BPEMER-PPEBP2-GMOT-0MOTEUR</t>
+          <t>SF01-UT-00PC-PST60D</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>MOTEUR ELECTRIQUE MT</t>
+          <t>POSTE ELECTRIQUE 60KV SALLE DISJONCTEURS</t>
         </is>
       </c>
       <c r="G8" t="inlineStr"/>
       <c r="H8" t="inlineStr"/>
       <c r="I8" t="inlineStr">
         <is>
-          <t>S-PC-BP2-M</t>
+          <t>S-PC-POST-60KV-DSJ</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
@@ -1172,17 +1172,17 @@
         </is>
       </c>
       <c r="P8" s="2" t="n">
-        <v>46289</v>
+        <v>46292</v>
       </c>
       <c r="Q8" s="2" t="n">
         <v>46286</v>
       </c>
       <c r="R8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>OT exécution &lt;1 mois | Performance Inspection</t>
+          <t>OT exécution &lt;1 mois</t>
         </is>
       </c>
       <c r="T8" t="inlineStr">
@@ -1192,42 +1192,42 @@
       </c>
       <c r="U8" t="inlineStr">
         <is>
-          <t>Exécuter les ordres lancés conformément au planning hebdomadaire validé. | Réaliser l'ensemble des inspections planifiées et consigner les anomalies détectées.</t>
+          <t>Exécuter les ordres lancés conformément au planning hebdomadaire validé.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>13737031</v>
+        <v>13736953</v>
       </c>
       <c r="B9" t="n">
-        <v>4002815932</v>
+        <v>4002815814</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Contrôle tableau BT en marche</t>
+          <t>Entretien systé salle électriq</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>OR004002815932</t>
+          <t>OR004002815814</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>SF01-UT-0PEM-POSTBT-00TGBT</t>
+          <t>SF01-UT-00PC-PST60R</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>TABLEAU ELECTRIQUE BASSE TENSION</t>
+          <t>POSTE ELECTRIQUE 60KV SALLE RELAIS</t>
         </is>
       </c>
       <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr"/>
       <c r="I9" t="inlineStr">
         <is>
-          <t>S-PC-TGBT-PEM</t>
+          <t>S-PC-POST-60KV-RL</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
@@ -1261,27 +1261,2252 @@
         </is>
       </c>
       <c r="P9" s="2" t="n">
-        <v>46289</v>
+        <v>46292</v>
       </c>
       <c r="Q9" s="2" t="n">
         <v>46286</v>
       </c>
       <c r="R9" t="n">
+        <v>1</v>
+      </c>
+      <c r="S9" t="inlineStr">
+        <is>
+          <t>OT exécution &lt;1 mois</t>
+        </is>
+      </c>
+      <c r="T9" t="inlineStr">
+        <is>
+          <t>Chef d'Atelier</t>
+        </is>
+      </c>
+      <c r="U9" t="inlineStr">
+        <is>
+          <t>Exécuter les ordres lancés conformément au planning hebdomadaire validé.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>13736954</v>
+      </c>
+      <c r="B10" t="n">
+        <v>4002815815</v>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Entretien systé salle électriq</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>OR004002815815</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>SF01-UT-00PC-PSTBTR</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>POSTE ELECTRIQUE BATTERIES NC MC</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr"/>
+      <c r="H10" t="inlineStr"/>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>S-PC-POST-BAT-PC</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>SF1-ECU</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>GM7</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>SF01</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>LANC CCRP PART RIMP TEC  TàLT</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>SOPL</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>IP1020260921</t>
+        </is>
+      </c>
+      <c r="P10" s="2" t="n">
+        <v>46292</v>
+      </c>
+      <c r="Q10" s="2" t="n">
+        <v>46286</v>
+      </c>
+      <c r="R10" t="n">
+        <v>1</v>
+      </c>
+      <c r="S10" t="inlineStr">
+        <is>
+          <t>OT exécution &lt;1 mois</t>
+        </is>
+      </c>
+      <c r="T10" t="inlineStr">
+        <is>
+          <t>Chef d'Atelier</t>
+        </is>
+      </c>
+      <c r="U10" t="inlineStr">
+        <is>
+          <t>Exécuter les ordres lancés conformément au planning hebdomadaire validé.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>13736956</v>
+      </c>
+      <c r="B11" t="n">
+        <v>4002815817</v>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Entretien systé salle électriq</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>OR004002815817</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>SF01-UT-00PC-POSTBT</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>POSTE ELECTRIQUE BASSE TENSION</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr"/>
+      <c r="H11" t="inlineStr"/>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>S-PC-POST-BT-PC</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>SF1-ECU</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>GM7</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>SF01</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>LANC CCRP PART RIMP TEC  TàLT</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>SOPL</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>IP1020260921</t>
+        </is>
+      </c>
+      <c r="P11" s="2" t="n">
+        <v>46292</v>
+      </c>
+      <c r="Q11" s="2" t="n">
+        <v>46286</v>
+      </c>
+      <c r="R11" t="n">
+        <v>1</v>
+      </c>
+      <c r="S11" t="inlineStr">
+        <is>
+          <t>OT exécution &lt;1 mois</t>
+        </is>
+      </c>
+      <c r="T11" t="inlineStr">
+        <is>
+          <t>Chef d'Atelier</t>
+        </is>
+      </c>
+      <c r="U11" t="inlineStr">
+        <is>
+          <t>Exécuter les ordres lancés conformément au planning hebdomadaire validé.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>13736957</v>
+      </c>
+      <c r="B12" t="n">
+        <v>4002815818</v>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Entretien systé salle électriq</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>OR004002815818</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>SF01-PS-PS03-POSTBT</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>POSTE ELECTRIQUE BASSE TENSION</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr"/>
+      <c r="H12" t="inlineStr"/>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>S-PC-POST-BT-PSIII</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>SF1-ECU</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>GM7</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>SF01</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>LANC CCRP PART RIMP TEC  TàLT</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>SOPL</t>
+        </is>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>IP1020260921</t>
+        </is>
+      </c>
+      <c r="P12" s="2" t="n">
+        <v>46292</v>
+      </c>
+      <c r="Q12" s="2" t="n">
+        <v>46286</v>
+      </c>
+      <c r="R12" t="n">
+        <v>1</v>
+      </c>
+      <c r="S12" t="inlineStr">
+        <is>
+          <t>OT exécution &lt;1 mois</t>
+        </is>
+      </c>
+      <c r="T12" t="inlineStr">
+        <is>
+          <t>Chef d'Atelier</t>
+        </is>
+      </c>
+      <c r="U12" t="inlineStr">
+        <is>
+          <t>Exécuter les ordres lancés conformément au planning hebdomadaire validé.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>13736947</v>
+      </c>
+      <c r="B13" t="n">
+        <v>4002815828</v>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Control hebdomadaire post élec</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>OR004002815828</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>SF01-UT-0TED-000CP5-POSTBT</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>POSTE ELECTRIQUE BASSE TENSION</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr"/>
+      <c r="H13" t="inlineStr"/>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>S-PC-POST-BT-CP5</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>SF1-ECU</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>GM7</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>SF01</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>LANC CCRP PART RIMP TEC  TàLT</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>SOPL</t>
+        </is>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>IP1020260921</t>
+        </is>
+      </c>
+      <c r="P13" s="2" t="n">
+        <v>46292</v>
+      </c>
+      <c r="Q13" s="2" t="n">
+        <v>46286</v>
+      </c>
+      <c r="R13" t="n">
+        <v>1</v>
+      </c>
+      <c r="S13" t="inlineStr">
+        <is>
+          <t>OT exécution &lt;1 mois</t>
+        </is>
+      </c>
+      <c r="T13" t="inlineStr">
+        <is>
+          <t>Chef d'Atelier</t>
+        </is>
+      </c>
+      <c r="U13" t="inlineStr">
+        <is>
+          <t>Exécuter les ordres lancés conformément au planning hebdomadaire validé.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>13736948</v>
+      </c>
+      <c r="B14" t="n">
+        <v>4002815829</v>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Control hebdomadaire post élec</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>OR004002815829</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>SF01-UT-0TED-000CP6-POSTBT</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>POSTE ELECTRIQUE BASSE TENSION</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr"/>
+      <c r="H14" t="inlineStr"/>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>S-PC-POST-BT-CP6</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>SF1-ECU</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>GM7</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>SF01</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>LANC CCRP PART RIMP TEC  TàLT</t>
+        </is>
+      </c>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>SOPL</t>
+        </is>
+      </c>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>IP1020260921</t>
+        </is>
+      </c>
+      <c r="P14" s="2" t="n">
+        <v>46292</v>
+      </c>
+      <c r="Q14" s="2" t="n">
+        <v>46286</v>
+      </c>
+      <c r="R14" t="n">
+        <v>1</v>
+      </c>
+      <c r="S14" t="inlineStr">
+        <is>
+          <t>OT exécution &lt;1 mois</t>
+        </is>
+      </c>
+      <c r="T14" t="inlineStr">
+        <is>
+          <t>Chef d'Atelier</t>
+        </is>
+      </c>
+      <c r="U14" t="inlineStr">
+        <is>
+          <t>Exécuter les ordres lancés conformément au planning hebdomadaire validé.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>13736949</v>
+      </c>
+      <c r="B15" t="n">
+        <v>4002815830</v>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Control hebdomadaire post élec</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>OR004002815830</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>SF01-UT-0TED-PSTMBT</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>POSTE ELECTRIQUE MT BT</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr"/>
+      <c r="H15" t="inlineStr"/>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>S-PC-POST-MTBT-TED</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>SF1-ECU</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>GM7</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>SF01</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>LANC CCRP PART RIMP TEC  TàLT</t>
+        </is>
+      </c>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>SOPL</t>
+        </is>
+      </c>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>IP1020260921</t>
+        </is>
+      </c>
+      <c r="P15" s="2" t="n">
+        <v>46292</v>
+      </c>
+      <c r="Q15" s="2" t="n">
+        <v>46286</v>
+      </c>
+      <c r="R15" t="n">
+        <v>1</v>
+      </c>
+      <c r="S15" t="inlineStr">
+        <is>
+          <t>OT exécution &lt;1 mois</t>
+        </is>
+      </c>
+      <c r="T15" t="inlineStr">
+        <is>
+          <t>Chef d'Atelier</t>
+        </is>
+      </c>
+      <c r="U15" t="inlineStr">
+        <is>
+          <t>Exécuter les ordres lancés conformément au planning hebdomadaire validé.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>13736959</v>
+      </c>
+      <c r="B16" t="n">
+        <v>4002815860</v>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Entretien systé salle électriq</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>OR004002815860</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>SF01-UT-00PC-PSTEXC</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>POSTE ELECTRIQUE EXCITATION GTA NC MC</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr"/>
+      <c r="H16" t="inlineStr"/>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>S-PC-POST-EXC-PC</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>SF1-ECU</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>GM7</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>SF01</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>LANC CCRP PART RIMP TEC  TàLT</t>
+        </is>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>SOPL</t>
+        </is>
+      </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>IP1020260921</t>
+        </is>
+      </c>
+      <c r="P16" s="2" t="n">
+        <v>46292</v>
+      </c>
+      <c r="Q16" s="2" t="n">
+        <v>46286</v>
+      </c>
+      <c r="R16" t="n">
+        <v>1</v>
+      </c>
+      <c r="S16" t="inlineStr">
+        <is>
+          <t>OT exécution &lt;1 mois</t>
+        </is>
+      </c>
+      <c r="T16" t="inlineStr">
+        <is>
+          <t>Chef d'Atelier</t>
+        </is>
+      </c>
+      <c r="U16" t="inlineStr">
+        <is>
+          <t>Exécuter les ordres lancés conformément au planning hebdomadaire validé.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>13736961</v>
+      </c>
+      <c r="B17" t="n">
+        <v>4002815862</v>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Entretien systé salle électriq</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>OR004002815862</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>SF01-UT-00PC-POSTMT</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>POSTE ELECTRIQUE MOYENNE TENSION</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr"/>
+      <c r="H17" t="inlineStr"/>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>S-PC-POST-MT-PC</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>SF1-ECU</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>GM7</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>SF01</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>LANC CCRP PART RIMP TEC  TàLT</t>
+        </is>
+      </c>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>SOPL</t>
+        </is>
+      </c>
+      <c r="O17" t="inlineStr">
+        <is>
+          <t>IP1020260921</t>
+        </is>
+      </c>
+      <c r="P17" s="2" t="n">
+        <v>46292</v>
+      </c>
+      <c r="Q17" s="2" t="n">
+        <v>46286</v>
+      </c>
+      <c r="R17" t="n">
+        <v>1</v>
+      </c>
+      <c r="S17" t="inlineStr">
+        <is>
+          <t>OT exécution &lt;1 mois</t>
+        </is>
+      </c>
+      <c r="T17" t="inlineStr">
+        <is>
+          <t>Chef d'Atelier</t>
+        </is>
+      </c>
+      <c r="U17" t="inlineStr">
+        <is>
+          <t>Exécuter les ordres lancés conformément au planning hebdomadaire validé.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>13736964</v>
+      </c>
+      <c r="B18" t="n">
+        <v>4002815865</v>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Entretien systé salle électriq</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>OR004002815865</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>SF01-PS-PS03-POSTMT</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>POSTE ELECTRIQUE MOYENNE TENSION</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr"/>
+      <c r="H18" t="inlineStr"/>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>S-PC-POST-MT-PSIII</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>SF1-ECU</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>GM7</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>SF01</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>LANC CCRP PART RIMP TEC  TàLT</t>
+        </is>
+      </c>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>SOPL</t>
+        </is>
+      </c>
+      <c r="O18" t="inlineStr">
+        <is>
+          <t>IP1020260921</t>
+        </is>
+      </c>
+      <c r="P18" s="2" t="n">
+        <v>46292</v>
+      </c>
+      <c r="Q18" s="2" t="n">
+        <v>46286</v>
+      </c>
+      <c r="R18" t="n">
+        <v>1</v>
+      </c>
+      <c r="S18" t="inlineStr">
+        <is>
+          <t>OT exécution &lt;1 mois</t>
+        </is>
+      </c>
+      <c r="T18" t="inlineStr">
+        <is>
+          <t>Chef d'Atelier</t>
+        </is>
+      </c>
+      <c r="U18" t="inlineStr">
+        <is>
+          <t>Exécuter les ordres lancés conformément au planning hebdomadaire validé.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>13736967</v>
+      </c>
+      <c r="B19" t="n">
+        <v>4002815868</v>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Entretien systé salle électriq</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>OR004002815868</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>SF01-UT-00PC-PSTOND</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>POSTE ELECTRIQUE ONDULEUR NC MC</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr"/>
+      <c r="H19" t="inlineStr"/>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>S-PC-POST-OND-PC</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>SF1-ECU</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>GM7</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>SF01</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>LANC CCRP PART RIMP TEC  TàLT</t>
+        </is>
+      </c>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>SOPL</t>
+        </is>
+      </c>
+      <c r="O19" t="inlineStr">
+        <is>
+          <t>IP1020260921</t>
+        </is>
+      </c>
+      <c r="P19" s="2" t="n">
+        <v>46292</v>
+      </c>
+      <c r="Q19" s="2" t="n">
+        <v>46286</v>
+      </c>
+      <c r="R19" t="n">
+        <v>1</v>
+      </c>
+      <c r="S19" t="inlineStr">
+        <is>
+          <t>OT exécution &lt;1 mois</t>
+        </is>
+      </c>
+      <c r="T19" t="inlineStr">
+        <is>
+          <t>Chef d'Atelier</t>
+        </is>
+      </c>
+      <c r="U19" t="inlineStr">
+        <is>
+          <t>Exécuter les ordres lancés conformément au planning hebdomadaire validé.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>13736970</v>
+      </c>
+      <c r="B20" t="n">
+        <v>4002815871</v>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Entretien systé salle électriq</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>OR004002815871</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>SF01-PS-PS03-PONDLU</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>POSTE ELECTRIQUE DES ONDULEURS</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr"/>
+      <c r="H20" t="inlineStr"/>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>S-PC-POST-OND-PSIII</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>SF1-ECU</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>GM7</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>SF01</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>LANC CCRP PART RIMP TEC  TàLT</t>
+        </is>
+      </c>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>SOPL</t>
+        </is>
+      </c>
+      <c r="O20" t="inlineStr">
+        <is>
+          <t>IP1020260921</t>
+        </is>
+      </c>
+      <c r="P20" s="2" t="n">
+        <v>46292</v>
+      </c>
+      <c r="Q20" s="2" t="n">
+        <v>46286</v>
+      </c>
+      <c r="R20" t="n">
+        <v>1</v>
+      </c>
+      <c r="S20" t="inlineStr">
+        <is>
+          <t>OT exécution &lt;1 mois</t>
+        </is>
+      </c>
+      <c r="T20" t="inlineStr">
+        <is>
+          <t>Chef d'Atelier</t>
+        </is>
+      </c>
+      <c r="U20" t="inlineStr">
+        <is>
+          <t>Exécuter les ordres lancés conformément au planning hebdomadaire validé.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>13737012</v>
+      </c>
+      <c r="B21" t="n">
+        <v>4002815913</v>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Test hebdomadair groupe diesel</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>OR004002815913</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>SF01-UT-00PC-FACIEL-000GES</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>GROUPE DIESEL DE SECOURS GES 2MW</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr"/>
+      <c r="H21" t="inlineStr"/>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>S-PC-GES</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>SF1-ECU</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>GM7</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>SF01</t>
+        </is>
+      </c>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>LANC CCRP PART RIMP TEC  TàLT</t>
+        </is>
+      </c>
+      <c r="N21" t="inlineStr">
+        <is>
+          <t>SOPL</t>
+        </is>
+      </c>
+      <c r="O21" t="inlineStr">
+        <is>
+          <t>IP1020260921</t>
+        </is>
+      </c>
+      <c r="P21" s="2" t="n">
+        <v>46292</v>
+      </c>
+      <c r="Q21" s="2" t="n">
+        <v>46286</v>
+      </c>
+      <c r="R21" t="n">
+        <v>1</v>
+      </c>
+      <c r="S21" t="inlineStr">
+        <is>
+          <t>OT exécution &lt;1 mois</t>
+        </is>
+      </c>
+      <c r="T21" t="inlineStr">
+        <is>
+          <t>Chef d'Atelier</t>
+        </is>
+      </c>
+      <c r="U21" t="inlineStr">
+        <is>
+          <t>Exécuter les ordres lancés conformément au planning hebdomadaire validé.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>13737018</v>
+      </c>
+      <c r="B22" t="n">
+        <v>4002815919</v>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Insp syst (7jours) TR HT 30MVA</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>OR004002815919</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>SF01-UT-00PC-PSTTRH-00TRHT</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>TRANSFORMATEUR HAUTE TENSION 30MVA</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr"/>
+      <c r="H22" t="inlineStr"/>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>S-PC-30MVA-T</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>SF1-ECU</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>GM7</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>SF01</t>
+        </is>
+      </c>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>LANC CCRP PART RIMP TEC  TàLT</t>
+        </is>
+      </c>
+      <c r="N22" t="inlineStr">
+        <is>
+          <t>SOPL</t>
+        </is>
+      </c>
+      <c r="O22" t="inlineStr">
+        <is>
+          <t>IP1020260921</t>
+        </is>
+      </c>
+      <c r="P22" s="2" t="n">
+        <v>46292</v>
+      </c>
+      <c r="Q22" s="2" t="n">
+        <v>46286</v>
+      </c>
+      <c r="R22" t="n">
+        <v>1</v>
+      </c>
+      <c r="S22" t="inlineStr">
+        <is>
+          <t>OT exécution &lt;1 mois</t>
+        </is>
+      </c>
+      <c r="T22" t="inlineStr">
+        <is>
+          <t>Chef d'Atelier</t>
+        </is>
+      </c>
+      <c r="U22" t="inlineStr">
+        <is>
+          <t>Exécuter les ordres lancés conformément au planning hebdomadaire validé.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>13737020</v>
+      </c>
+      <c r="B23" t="n">
+        <v>4002815921</v>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>inspection Postes électriques</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>OR004002815921</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>SF01-UT-00PC-PST60D</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>POSTE ELECTRIQUE 60KV SALLE DISJONCTEURS</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr"/>
+      <c r="H23" t="inlineStr"/>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>S-PC-POST-60KV-DSJ</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>SF1-ECU</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>GM7</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>SF01</t>
+        </is>
+      </c>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>LANC CCRP PART RIMP TEC  TàLT</t>
+        </is>
+      </c>
+      <c r="N23" t="inlineStr">
+        <is>
+          <t>SOPL</t>
+        </is>
+      </c>
+      <c r="O23" t="inlineStr">
+        <is>
+          <t>IP1020260921</t>
+        </is>
+      </c>
+      <c r="P23" s="2" t="n">
+        <v>46292</v>
+      </c>
+      <c r="Q23" s="2" t="n">
+        <v>46286</v>
+      </c>
+      <c r="R23" t="n">
+        <v>1</v>
+      </c>
+      <c r="S23" t="inlineStr">
+        <is>
+          <t>OT exécution &lt;1 mois</t>
+        </is>
+      </c>
+      <c r="T23" t="inlineStr">
+        <is>
+          <t>Chef d'Atelier</t>
+        </is>
+      </c>
+      <c r="U23" t="inlineStr">
+        <is>
+          <t>Exécuter les ordres lancés conformément au planning hebdomadaire validé.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>13737022</v>
+      </c>
+      <c r="B24" t="n">
+        <v>4002815923</v>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>inspection Postes électriques</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>OR004002815923</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>SF01-UT-00PC-PST60R</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>POSTE ELECTRIQUE 60KV SALLE RELAIS</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr"/>
+      <c r="H24" t="inlineStr"/>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>S-PC-POST-60KV-RL</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>SF1-ECU</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>GM7</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>SF01</t>
+        </is>
+      </c>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>LANC CCRP PART RIMP TEC  TàLT</t>
+        </is>
+      </c>
+      <c r="N24" t="inlineStr">
+        <is>
+          <t>SOPL</t>
+        </is>
+      </c>
+      <c r="O24" t="inlineStr">
+        <is>
+          <t>IP1020260921</t>
+        </is>
+      </c>
+      <c r="P24" s="2" t="n">
+        <v>46292</v>
+      </c>
+      <c r="Q24" s="2" t="n">
+        <v>46286</v>
+      </c>
+      <c r="R24" t="n">
+        <v>1</v>
+      </c>
+      <c r="S24" t="inlineStr">
+        <is>
+          <t>OT exécution &lt;1 mois</t>
+        </is>
+      </c>
+      <c r="T24" t="inlineStr">
+        <is>
+          <t>Chef d'Atelier</t>
+        </is>
+      </c>
+      <c r="U24" t="inlineStr">
+        <is>
+          <t>Exécuter les ordres lancés conformément au planning hebdomadaire validé.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>13737023</v>
+      </c>
+      <c r="B25" t="n">
+        <v>4002815925</v>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Contrôle moteur MT en marche</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>OR004002815925</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>SF01-UT-0PEM-BPEMER-PPEBP2-GMOT-0MOTEUR</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>MOTEUR ELECTRIQUE MT</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr"/>
+      <c r="H25" t="inlineStr"/>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>S-PC-BP2-M</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>SF1-ECU</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>GM7</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>SF01</t>
+        </is>
+      </c>
+      <c r="M25" t="inlineStr">
+        <is>
+          <t>LANC CCRP PART RIMP TEC  TàLT</t>
+        </is>
+      </c>
+      <c r="N25" t="inlineStr">
+        <is>
+          <t>SOPL</t>
+        </is>
+      </c>
+      <c r="O25" t="inlineStr">
+        <is>
+          <t>IP1020260921</t>
+        </is>
+      </c>
+      <c r="P25" s="2" t="n">
+        <v>46289</v>
+      </c>
+      <c r="Q25" s="2" t="n">
+        <v>46286</v>
+      </c>
+      <c r="R25" t="n">
         <v>2</v>
       </c>
-      <c r="S9" t="inlineStr">
+      <c r="S25" t="inlineStr">
         <is>
           <t>OT exécution &lt;1 mois | Performance Inspection</t>
         </is>
       </c>
-      <c r="T9" t="inlineStr">
+      <c r="T25" t="inlineStr">
         <is>
           <t>Chef d'Atelier</t>
         </is>
       </c>
-      <c r="U9" t="inlineStr">
+      <c r="U25" t="inlineStr">
         <is>
           <t>Exécuter les ordres lancés conformément au planning hebdomadaire validé. | Réaliser l'ensemble des inspections planifiées et consigner les anomalies détectées.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>13737027</v>
+      </c>
+      <c r="B26" t="n">
+        <v>4002815928</v>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>inspection Postes électriques</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>OR004002815928</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>SF01-UT-00PC-PSTBTR</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>POSTE ELECTRIQUE BATTERIES NC MC</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr"/>
+      <c r="H26" t="inlineStr"/>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>S-PC-POST-BAT-PC</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>SF1-ECU</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>GM7</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>SF01</t>
+        </is>
+      </c>
+      <c r="M26" t="inlineStr">
+        <is>
+          <t>LANC CCRP PART RIMP TEC  TàLT</t>
+        </is>
+      </c>
+      <c r="N26" t="inlineStr">
+        <is>
+          <t>SOPL</t>
+        </is>
+      </c>
+      <c r="O26" t="inlineStr">
+        <is>
+          <t>IP1020260921</t>
+        </is>
+      </c>
+      <c r="P26" s="2" t="n">
+        <v>46292</v>
+      </c>
+      <c r="Q26" s="2" t="n">
+        <v>46286</v>
+      </c>
+      <c r="R26" t="n">
+        <v>1</v>
+      </c>
+      <c r="S26" t="inlineStr">
+        <is>
+          <t>OT exécution &lt;1 mois</t>
+        </is>
+      </c>
+      <c r="T26" t="inlineStr">
+        <is>
+          <t>Chef d'Atelier</t>
+        </is>
+      </c>
+      <c r="U26" t="inlineStr">
+        <is>
+          <t>Exécuter les ordres lancés conformément au planning hebdomadaire validé.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>13737031</v>
+      </c>
+      <c r="B27" t="n">
+        <v>4002815932</v>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Contrôle tableau BT en marche</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>OR004002815932</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>SF01-UT-0PEM-POSTBT-00TGBT</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>TABLEAU ELECTRIQUE BASSE TENSION</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr"/>
+      <c r="H27" t="inlineStr"/>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>S-PC-TGBT-PEM</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>SF1-ECU</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>GM7</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>SF01</t>
+        </is>
+      </c>
+      <c r="M27" t="inlineStr">
+        <is>
+          <t>LANC CCRP PART RIMP TEC  TàLT</t>
+        </is>
+      </c>
+      <c r="N27" t="inlineStr">
+        <is>
+          <t>SOPL</t>
+        </is>
+      </c>
+      <c r="O27" t="inlineStr">
+        <is>
+          <t>IP1020260921</t>
+        </is>
+      </c>
+      <c r="P27" s="2" t="n">
+        <v>46289</v>
+      </c>
+      <c r="Q27" s="2" t="n">
+        <v>46286</v>
+      </c>
+      <c r="R27" t="n">
+        <v>2</v>
+      </c>
+      <c r="S27" t="inlineStr">
+        <is>
+          <t>OT exécution &lt;1 mois | Performance Inspection</t>
+        </is>
+      </c>
+      <c r="T27" t="inlineStr">
+        <is>
+          <t>Chef d'Atelier</t>
+        </is>
+      </c>
+      <c r="U27" t="inlineStr">
+        <is>
+          <t>Exécuter les ordres lancés conformément au planning hebdomadaire validé. | Réaliser l'ensemble des inspections planifiées et consigner les anomalies détectées.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>13737032</v>
+      </c>
+      <c r="B28" t="n">
+        <v>4002815933</v>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>inspection Postes électriques</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>OR004002815933</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>SF01-UT-00PC-POSTBT</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>POSTE ELECTRIQUE BASSE TENSION</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr"/>
+      <c r="H28" t="inlineStr"/>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>S-PC-POST-BT-PC</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>SF1-ECU</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>GM7</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>SF01</t>
+        </is>
+      </c>
+      <c r="M28" t="inlineStr">
+        <is>
+          <t>LANC CCRP PART RIMP TEC  TàLT</t>
+        </is>
+      </c>
+      <c r="N28" t="inlineStr">
+        <is>
+          <t>SOPL</t>
+        </is>
+      </c>
+      <c r="O28" t="inlineStr">
+        <is>
+          <t>IP1020260921</t>
+        </is>
+      </c>
+      <c r="P28" s="2" t="n">
+        <v>46292</v>
+      </c>
+      <c r="Q28" s="2" t="n">
+        <v>46286</v>
+      </c>
+      <c r="R28" t="n">
+        <v>1</v>
+      </c>
+      <c r="S28" t="inlineStr">
+        <is>
+          <t>OT exécution &lt;1 mois</t>
+        </is>
+      </c>
+      <c r="T28" t="inlineStr">
+        <is>
+          <t>Chef d'Atelier</t>
+        </is>
+      </c>
+      <c r="U28" t="inlineStr">
+        <is>
+          <t>Exécuter les ordres lancés conformément au planning hebdomadaire validé.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>13737038</v>
+      </c>
+      <c r="B29" t="n">
+        <v>4002815938</v>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>inspection Postes électriques</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>OR004002815938</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>SF01-PS-PS03-POSTBT</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>POSTE ELECTRIQUE BASSE TENSION</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr"/>
+      <c r="H29" t="inlineStr"/>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>S-PC-POST-BT-PSIII</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>SF1-ECU</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>GM7</t>
+        </is>
+      </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>SF01</t>
+        </is>
+      </c>
+      <c r="M29" t="inlineStr">
+        <is>
+          <t>LANC CCRP PART RIMP TEC  TàLT</t>
+        </is>
+      </c>
+      <c r="N29" t="inlineStr">
+        <is>
+          <t>SOPL</t>
+        </is>
+      </c>
+      <c r="O29" t="inlineStr">
+        <is>
+          <t>IP1020260921</t>
+        </is>
+      </c>
+      <c r="P29" s="2" t="n">
+        <v>46292</v>
+      </c>
+      <c r="Q29" s="2" t="n">
+        <v>46286</v>
+      </c>
+      <c r="R29" t="n">
+        <v>1</v>
+      </c>
+      <c r="S29" t="inlineStr">
+        <is>
+          <t>OT exécution &lt;1 mois</t>
+        </is>
+      </c>
+      <c r="T29" t="inlineStr">
+        <is>
+          <t>Chef d'Atelier</t>
+        </is>
+      </c>
+      <c r="U29" t="inlineStr">
+        <is>
+          <t>Exécuter les ordres lancés conformément au planning hebdomadaire validé.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>13737043</v>
+      </c>
+      <c r="B30" t="n">
+        <v>4002815944</v>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>inspection Postes électriques</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>OR004002815944</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>SF01-UT-00PC-PSTEXC</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>POSTE ELECTRIQUE EXCITATION GTA NC MC</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr"/>
+      <c r="H30" t="inlineStr"/>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>S-PC-POST-EXC-PC</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>SF1-ECU</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>GM7</t>
+        </is>
+      </c>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>SF01</t>
+        </is>
+      </c>
+      <c r="M30" t="inlineStr">
+        <is>
+          <t>LANC CCRP PART RIMP TEC  TàLT</t>
+        </is>
+      </c>
+      <c r="N30" t="inlineStr">
+        <is>
+          <t>SOPL</t>
+        </is>
+      </c>
+      <c r="O30" t="inlineStr">
+        <is>
+          <t>IP1020260921</t>
+        </is>
+      </c>
+      <c r="P30" s="2" t="n">
+        <v>46292</v>
+      </c>
+      <c r="Q30" s="2" t="n">
+        <v>46286</v>
+      </c>
+      <c r="R30" t="n">
+        <v>1</v>
+      </c>
+      <c r="S30" t="inlineStr">
+        <is>
+          <t>OT exécution &lt;1 mois</t>
+        </is>
+      </c>
+      <c r="T30" t="inlineStr">
+        <is>
+          <t>Chef d'Atelier</t>
+        </is>
+      </c>
+      <c r="U30" t="inlineStr">
+        <is>
+          <t>Exécuter les ordres lancés conformément au planning hebdomadaire validé.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>13737046</v>
+      </c>
+      <c r="B31" t="n">
+        <v>4002815947</v>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>inspection Postes électriques</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>OR004002815947</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>SF01-UT-00PC-POSTMT</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>POSTE ELECTRIQUE MOYENNE TENSION</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr"/>
+      <c r="H31" t="inlineStr"/>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>S-PC-POST-MT-PC</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>SF1-ECU</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>GM7</t>
+        </is>
+      </c>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>SF01</t>
+        </is>
+      </c>
+      <c r="M31" t="inlineStr">
+        <is>
+          <t>LANC CCRP PART RIMP TEC  TàLT</t>
+        </is>
+      </c>
+      <c r="N31" t="inlineStr">
+        <is>
+          <t>SOPL</t>
+        </is>
+      </c>
+      <c r="O31" t="inlineStr">
+        <is>
+          <t>IP1020260921</t>
+        </is>
+      </c>
+      <c r="P31" s="2" t="n">
+        <v>46292</v>
+      </c>
+      <c r="Q31" s="2" t="n">
+        <v>46286</v>
+      </c>
+      <c r="R31" t="n">
+        <v>1</v>
+      </c>
+      <c r="S31" t="inlineStr">
+        <is>
+          <t>OT exécution &lt;1 mois</t>
+        </is>
+      </c>
+      <c r="T31" t="inlineStr">
+        <is>
+          <t>Chef d'Atelier</t>
+        </is>
+      </c>
+      <c r="U31" t="inlineStr">
+        <is>
+          <t>Exécuter les ordres lancés conformément au planning hebdomadaire validé.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="n">
+        <v>13737051</v>
+      </c>
+      <c r="B32" t="n">
+        <v>4002815952</v>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>inspection Postes électriques</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>OR004002815952</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>SF01-PS-PS03-POSTMT</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>POSTE ELECTRIQUE MOYENNE TENSION</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr"/>
+      <c r="H32" t="inlineStr"/>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>S-PC-POST-MT-PSIII</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>SF1-ECU</t>
+        </is>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>GM7</t>
+        </is>
+      </c>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>SF01</t>
+        </is>
+      </c>
+      <c r="M32" t="inlineStr">
+        <is>
+          <t>LANC CCRP PART RIMP TEC  TàLT</t>
+        </is>
+      </c>
+      <c r="N32" t="inlineStr">
+        <is>
+          <t>SOPL</t>
+        </is>
+      </c>
+      <c r="O32" t="inlineStr">
+        <is>
+          <t>IP1020260921</t>
+        </is>
+      </c>
+      <c r="P32" s="2" t="n">
+        <v>46292</v>
+      </c>
+      <c r="Q32" s="2" t="n">
+        <v>46286</v>
+      </c>
+      <c r="R32" t="n">
+        <v>1</v>
+      </c>
+      <c r="S32" t="inlineStr">
+        <is>
+          <t>OT exécution &lt;1 mois</t>
+        </is>
+      </c>
+      <c r="T32" t="inlineStr">
+        <is>
+          <t>Chef d'Atelier</t>
+        </is>
+      </c>
+      <c r="U32" t="inlineStr">
+        <is>
+          <t>Exécuter les ordres lancés conformément au planning hebdomadaire validé.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="n">
+        <v>13737055</v>
+      </c>
+      <c r="B33" t="n">
+        <v>4002815956</v>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>inspection Postes électriques</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>OR004002815956</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>SF01-UT-00PC-PSTOND</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>POSTE ELECTRIQUE ONDULEUR NC MC</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr"/>
+      <c r="H33" t="inlineStr"/>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>S-PC-POST-OND-PC</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>SF1-ECU</t>
+        </is>
+      </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>GM7</t>
+        </is>
+      </c>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t>SF01</t>
+        </is>
+      </c>
+      <c r="M33" t="inlineStr">
+        <is>
+          <t>LANC CCRP PART RIMP TEC  TàLT</t>
+        </is>
+      </c>
+      <c r="N33" t="inlineStr">
+        <is>
+          <t>SOPL</t>
+        </is>
+      </c>
+      <c r="O33" t="inlineStr">
+        <is>
+          <t>IP1020260921</t>
+        </is>
+      </c>
+      <c r="P33" s="2" t="n">
+        <v>46292</v>
+      </c>
+      <c r="Q33" s="2" t="n">
+        <v>46286</v>
+      </c>
+      <c r="R33" t="n">
+        <v>1</v>
+      </c>
+      <c r="S33" t="inlineStr">
+        <is>
+          <t>OT exécution &lt;1 mois</t>
+        </is>
+      </c>
+      <c r="T33" t="inlineStr">
+        <is>
+          <t>Chef d'Atelier</t>
+        </is>
+      </c>
+      <c r="U33" t="inlineStr">
+        <is>
+          <t>Exécuter les ordres lancés conformément au planning hebdomadaire validé.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>13737059</v>
+      </c>
+      <c r="B34" t="n">
+        <v>4002815960</v>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>inspection Postes électriques</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>OR004002815960</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>SF01-PS-PS03-PONDLU</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>POSTE ELECTRIQUE DES ONDULEURS</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr"/>
+      <c r="H34" t="inlineStr"/>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>S-PC-POST-OND-PSIII</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>SF1-ECU</t>
+        </is>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>GM7</t>
+        </is>
+      </c>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>SF01</t>
+        </is>
+      </c>
+      <c r="M34" t="inlineStr">
+        <is>
+          <t>LANC CCRP PART RIMP TEC  TàLT</t>
+        </is>
+      </c>
+      <c r="N34" t="inlineStr">
+        <is>
+          <t>SOPL</t>
+        </is>
+      </c>
+      <c r="O34" t="inlineStr">
+        <is>
+          <t>IP1020260921</t>
+        </is>
+      </c>
+      <c r="P34" s="2" t="n">
+        <v>46292</v>
+      </c>
+      <c r="Q34" s="2" t="n">
+        <v>46286</v>
+      </c>
+      <c r="R34" t="n">
+        <v>1</v>
+      </c>
+      <c r="S34" t="inlineStr">
+        <is>
+          <t>OT exécution &lt;1 mois</t>
+        </is>
+      </c>
+      <c r="T34" t="inlineStr">
+        <is>
+          <t>Chef d'Atelier</t>
+        </is>
+      </c>
+      <c r="U34" t="inlineStr">
+        <is>
+          <t>Exécuter les ordres lancés conformément au planning hebdomadaire validé.</t>
         </is>
       </c>
     </row>

</xml_diff>